<commit_message>
updated flight data v2
</commit_message>
<xml_diff>
--- a/data/flight/growth/Ecoli_BC_LSMMG_1B.xlsx
+++ b/data/flight/growth/Ecoli_BC_LSMMG_1B.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cocoa\OneDrive\Desktop\HARV\processed ALL and flight data Feb 2024\Flight 1B\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ipjos\code\DARPA_FINAL\data\flight_uploaded_to_github_with_96_hours\growth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7670CCF1-6C95-4CBD-A0CE-75535FB05BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F07CD1-93FA-4ADF-99BA-AA7480EF8018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="26385" windowHeight="14250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="growth" sheetId="1" r:id="rId1"/>
@@ -170,61 +170,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -510,12 +462,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="13.5546875" customWidth="1"/>
+    <col min="1" max="6" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -535,7 +487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -576,181 +528,144 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="B3" s="3">
-        <v>0.29899999999999999</v>
+        <v>0.23200000000000001</v>
       </c>
       <c r="C3" s="3">
-        <v>0.31</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="D3" s="3">
-        <v>0.31</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="E3" s="3">
+        <v>0.27800000000000002</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.28199999999999997</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.27400000000000002</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="K3" s="3">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0.26900000000000002</v>
+      </c>
+      <c r="M3" s="3">
+        <v>0.26</v>
+      </c>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3">
+        <v>0.27100000000000002</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>0.23699999999999999</v>
+      </c>
+      <c r="AC3" s="3">
         <v>0.24299999999999999</v>
       </c>
-      <c r="F3" s="3">
-        <v>0.32500000000000001</v>
-      </c>
-      <c r="G3" s="3">
-        <v>0.31</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.28899999999999998</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0.29799999999999999</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="K3" s="3">
-        <v>0.33500000000000002</v>
-      </c>
-      <c r="L3" s="3">
-        <v>0.34200000000000003</v>
-      </c>
-      <c r="M3" s="3">
-        <v>0.33200000000000002</v>
-      </c>
-      <c r="N3" s="4">
-        <v>0.28799999999999998</v>
-      </c>
-      <c r="O3" s="4">
-        <v>0.28299999999999997</v>
-      </c>
-      <c r="P3" s="4">
-        <v>0.29899999999999999</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>0.26</v>
-      </c>
-      <c r="R3" s="5">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="S3" s="5">
-        <v>0.28199999999999997</v>
-      </c>
-      <c r="T3" s="6">
-        <v>0.27700000000000002</v>
-      </c>
-      <c r="U3" s="6">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="V3" s="6">
-        <v>0.28799999999999998</v>
-      </c>
-      <c r="W3" s="7">
-        <v>0.26800000000000002</v>
-      </c>
-      <c r="X3" s="7">
-        <v>0.27800000000000002</v>
-      </c>
-      <c r="Y3" s="7">
+      <c r="AD3" s="3">
+        <v>0.26500000000000001</v>
+      </c>
+      <c r="AE3" s="3">
+        <v>0.25900000000000001</v>
+      </c>
+      <c r="AF3" s="3">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AG3" s="3">
         <v>0.28599999999999998</v>
       </c>
-      <c r="Z3" s="12">
-        <v>0.26500000000000001</v>
-      </c>
-      <c r="AA3" s="12">
-        <v>0.27100000000000002</v>
-      </c>
-      <c r="AB3" s="12">
-        <v>0.23699999999999999</v>
-      </c>
-      <c r="AC3" s="13">
-        <v>0.24299999999999999</v>
-      </c>
-      <c r="AD3" s="13">
-        <v>0.26500000000000001</v>
-      </c>
-      <c r="AE3" s="13">
-        <v>0.25900000000000001</v>
-      </c>
-      <c r="AF3" s="14">
-        <v>0.27600000000000002</v>
-      </c>
-      <c r="AG3" s="14">
-        <v>0.28599999999999998</v>
-      </c>
-      <c r="AH3" s="14">
+      <c r="AH3" s="3">
         <v>0.30199999999999999</v>
       </c>
-      <c r="AI3" s="15">
+      <c r="AI3" s="3">
         <v>0.24099999999999999</v>
       </c>
-      <c r="AJ3" s="15">
+      <c r="AJ3" s="3">
         <v>0.24399999999999999</v>
       </c>
-      <c r="AK3" s="15">
+      <c r="AK3" s="3">
         <v>0.24199999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="E15" s="1"/>
     </row>
   </sheetData>
@@ -762,17 +677,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67820D14-AE55-4601-AB4D-CB8AD178327A}">
   <dimension ref="A1:AK13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="15.33203125" customWidth="1"/>
+    <col min="1" max="5" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -813,177 +728,115 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="B3" s="3">
-        <v>1.658263305322129</v>
+        <v>1.2324929971988794</v>
       </c>
       <c r="C3" s="3">
-        <v>1.5854341736694679</v>
+        <v>1.1120448179271707</v>
       </c>
       <c r="D3" s="3">
-        <v>1.596638655462185</v>
+        <v>1.0784313725490196</v>
       </c>
       <c r="E3" s="3">
-        <v>1.5826330532212887</v>
+        <v>1.1624649859943976</v>
       </c>
       <c r="F3" s="3">
-        <v>1.4733893557422968</v>
+        <v>1.3641456582633054</v>
       </c>
       <c r="G3" s="3">
-        <v>1.4313725490196076</v>
+        <v>1.187675070028011</v>
       </c>
       <c r="H3" s="3">
-        <v>1.6862745098039216</v>
+        <v>1.0840336134453781</v>
       </c>
       <c r="I3" s="3">
-        <v>1.7731092436974787</v>
+        <v>1.002801120448179</v>
       </c>
       <c r="J3" s="3">
-        <v>1.6946778711484594</v>
+        <v>0.94397759103641443</v>
       </c>
       <c r="K3" s="3">
-        <v>1.9243697478991595</v>
+        <v>1.1932773109243695</v>
       </c>
       <c r="L3" s="3">
-        <v>2.0280112044817931</v>
+        <v>1.1764705882352939</v>
       </c>
       <c r="M3" s="3">
-        <v>2.2016806722689077</v>
-      </c>
-      <c r="N3" s="8">
-        <v>1.0588235294117647</v>
-      </c>
-      <c r="O3" s="8">
-        <v>0.81792717086834732</v>
-      </c>
-      <c r="P3" s="8">
-        <v>0.81792717086834732</v>
-      </c>
-      <c r="Q3" s="9">
-        <v>0.81792717086834732</v>
-      </c>
-      <c r="R3" s="9">
-        <v>0.94397759103641443</v>
-      </c>
-      <c r="S3" s="9">
-        <v>0.89635854341736698</v>
-      </c>
-      <c r="T3" s="10">
-        <v>0.83193277310924363</v>
-      </c>
-      <c r="U3" s="10">
-        <v>0.85994397759103636</v>
-      </c>
-      <c r="V3" s="10">
-        <v>0.79271708683473396</v>
-      </c>
-      <c r="W3" s="11">
-        <v>0.90196078431372551</v>
-      </c>
-      <c r="X3" s="11">
-        <v>0.92717086834733886</v>
-      </c>
-      <c r="Y3" s="11">
-        <v>0.82352941176470584</v>
-      </c>
-      <c r="Z3" s="16">
-        <v>1.011204481792717</v>
-      </c>
-      <c r="AA3" s="16">
-        <v>1.072829131652661</v>
-      </c>
-      <c r="AB3" s="16">
-        <v>1.1120448179271707</v>
-      </c>
-      <c r="AC3" s="17">
-        <v>1.1652661064425769</v>
-      </c>
-      <c r="AD3" s="17">
-        <v>1.1764705882352939</v>
-      </c>
-      <c r="AE3" s="17">
-        <v>1.2156862745098038</v>
-      </c>
-      <c r="AF3" s="18">
-        <v>0.67787114845938368</v>
-      </c>
-      <c r="AG3" s="18">
-        <v>0.62745098039215674</v>
-      </c>
-      <c r="AH3" s="18">
-        <v>0.6162464985994397</v>
-      </c>
-      <c r="AI3" s="19">
         <v>1.2464985994397759</v>
       </c>
-      <c r="AJ3" s="19">
-        <v>1.0644257703081232</v>
-      </c>
-      <c r="AK3" s="19">
-        <v>1.1596638655462184</v>
-      </c>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3"/>
+    </row>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
   </sheetData>
@@ -994,12 +847,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9C5B29F-B2ED-4FDE-BD7E-A42BB3247F1C}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="44.6640625" customWidth="1"/>
+    <col min="1" max="4" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1007,7 +860,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1015,7 +868,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1023,7 +876,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1031,12 +884,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1044,7 +897,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>

</xml_diff>